<commit_message>
stable before chaning monthly
</commit_message>
<xml_diff>
--- a/Offlinereports/reports/Swornima Shakya_transactions.xlsx
+++ b/Offlinereports/reports/Swornima Shakya_transactions.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +457,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45827</v>
+        <v>45827.63045138889</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -465,47 +465,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>income</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>45827</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>needs</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>expense</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>45827</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>wants</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>expense</t>
         </is>
       </c>
     </row>
@@ -543,7 +507,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rs 5000.00</t>
+          <t>Rs 1000.00</t>
         </is>
       </c>
     </row>
@@ -555,7 +519,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rs 7000.00</t>
+          <t>Rs 0.00</t>
         </is>
       </c>
     </row>
@@ -567,7 +531,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Deficit: Rs 2000.00</t>
+          <t>Rs 1000.00</t>
         </is>
       </c>
     </row>
@@ -579,31 +543,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OVERSPENDING</t>
+          <t>HEALTHY</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Recommended Action</t>
+          <t>Expense Ratio</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Reduce expenses or increase income</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Expense Ratio</t>
+          <t>Savings Rate</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>140.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>

</xml_diff>